<commit_message>
Clarify M0 test direction; neutral analysis-plan notes; public source labels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_S3.xlsx
+++ b/supplementary_tables/Supplementary_Table_S3.xlsx
@@ -239,7 +239,7 @@
     <t xml:space="preserve">67,099</t>
   </si>
   <si>
-    <t xml:space="preserve">N28_fig/data/sc_umap.tsv.gz</t>
+    <t xml:space="preserve">figures/data/sc_umap.tsv.gz</t>
   </si>
   <si>
     <t xml:space="preserve">sc_patients</t>
@@ -269,7 +269,7 @@
     <t xml:space="preserve">50</t>
   </si>
   <si>
-    <t xml:space="preserve">N11_scripts/robust_proxy.R</t>
+    <t xml:space="preserve">analysis/robust_proxy.R</t>
   </si>
   <si>
     <t xml:space="preserve">N11_S default</t>

</xml_diff>

<commit_message>
Sync supplementary analyses and figure numbering
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_S3.xlsx
+++ b/supplementary_tables/Supplementary_Table_S3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="1038">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="1072">
   <si>
     <t xml:space="preserve">Supplementary Table S3. Every quantity reported in the text and figures, with source file and extraction rule.</t>
   </si>
@@ -989,7 +989,7 @@
     <t xml:space="preserve">C3_M13_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Immune checkpoint expression differs</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Immune checkpoint expression differs</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M15_rand</t>
@@ -1007,7 +1007,7 @@
     <t xml:space="preserve">C3_M15_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Decision curve shows net benefit</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Decision curve shows net benefit</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M3_rand</t>
@@ -1028,7 +1028,7 @@
     <t xml:space="preserve">C3_M3_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Drug sensitivity differs (oncoPredict)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Drug sensitivity differs (oncoPredict)</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M4_rand</t>
@@ -1046,7 +1046,7 @@
     <t xml:space="preserve">C3_M4_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, GSEA Hallmark pathways enriched</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, GSEA Hallmark pathways enriched</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M2_rand</t>
@@ -1067,7 +1067,7 @@
     <t xml:space="preserve">C3_M2_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Immune infiltration differs by risk group</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Immune infiltration differs by risk group</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M1_rand</t>
@@ -1091,7 +1091,7 @@
     <t xml:space="preserve">C3_M1_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Independent prognostic factor (multivariable Cox)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Independent prognostic factor (multivariable Cox)</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M5b_rand</t>
@@ -1115,7 +1115,7 @@
     <t xml:space="preserve">C3_M5b_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, TMB x risk groups separate survival</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, TMB x risk groups separate survival</t>
   </si>
   <si>
     <t xml:space="preserve">4.4e-31</t>
@@ -1142,7 +1142,7 @@
     <t xml:space="preserve">C3_M8b_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Signature genes differ tumour vs normal (scRNA)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Signature genes differ tumour vs normal (scRNA)</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M14_rand</t>
@@ -1166,7 +1166,7 @@
     <t xml:space="preserve">C3_M14_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Consensus-clustering subtypes differ in survival</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Consensus-clustering subtypes differ in survival</t>
   </si>
   <si>
     <t xml:space="preserve">2.7e-15</t>
@@ -1193,7 +1193,7 @@
     <t xml:space="preserve">C3_M7_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Multi-algorithm model selection</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Multi-algorithm model selection</t>
   </si>
   <si>
     <t xml:space="preserve">1.1e-04</t>
@@ -1220,7 +1220,7 @@
     <t xml:space="preserve">C3_M8a_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Signature genes mark a cell type (scRNA)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Signature genes mark a cell type (scRNA)</t>
   </si>
   <si>
     <t xml:space="preserve">0.021</t>
@@ -1247,7 +1247,7 @@
     <t xml:space="preserve">C3_M0_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, External validation (C &gt; 0.5, both cohorts)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, External validation (C &gt; 0.5, both cohorts)</t>
   </si>
   <si>
     <t xml:space="preserve">8.1e-04</t>
@@ -1274,7 +1274,7 @@
     <t xml:space="preserve">C3_M12_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Drugs enriched (DSigDB)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Drugs enriched (DSigDB)</t>
   </si>
   <si>
     <t xml:space="preserve">1.0e-05</t>
@@ -1301,7 +1301,7 @@
     <t xml:space="preserve">C3_M6_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Nomogram adds to stage (nested LRT)</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Nomogram adds to stage (nested LRT)</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M5a_rand</t>
@@ -1325,7 +1325,7 @@
     <t xml:space="preserve">C3_M5a_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, TMB differs by risk group</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, TMB differs by risk group</t>
   </si>
   <si>
     <t xml:space="preserve">C3_M10_rand</t>
@@ -1349,7 +1349,7 @@
     <t xml:space="preserve">C3_M10_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Fisher P published vs size-matched, Geneformer in silico deletion</t>
+    <t xml:space="preserve">Holm-adjusted stratified CMH P, published vs size-matched, Geneformer in silico deletion</t>
   </si>
   <si>
     <t xml:space="preserve">0.93</t>
@@ -2606,7 +2606,7 @@
     <t xml:space="preserve">S1_n_same_verdict</t>
   </si>
   <si>
-    <t xml:space="preserve">FigS1b</t>
+    <t xml:space="preserve">FigS4b</t>
   </si>
   <si>
     <t xml:space="preserve">Modules with same verdict at n = 148 and n = 95</t>
@@ -2681,31 +2681,139 @@
     <t xml:space="preserve">S4_top25_prolif</t>
   </si>
   <si>
+    <t xml:space="preserve">FigS1a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hallmark E2F/G2M genes among 25 most reused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5/25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS4a_gene_frequency.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">top 25 by n_sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4_top_gene_n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signatures containing G6PD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G6PD: 19 signatures, 5 death types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">top 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1_n_null_default</t>
+  </si>
+  <si>
     <t xml:space="preserve">FigS4a</t>
   </si>
   <si>
-    <t xml:space="preserve">Hallmark E2F/G2M genes among 25 most reused</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5/25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FigS4a_gene_frequency.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">top 25 by n_sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4_top_gene_n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signatures containing G6PD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G6PD: 19 signatures, 5 death types</t>
-  </si>
-  <si>
-    <t xml:space="preserve">top 1</t>
+    <t xml:space="preserve">Size-matched random signatures per module, full-coverage subset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,375</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS1a_fullcoverage_module_rates.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modal n_null</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1_n_null_M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size-matched random signatures, multi-algorithm module, full-coverage subset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 n_null</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1_n_null_M14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size-matched random signatures, consensus clustering, full-coverage subset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,308</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M14 n_null</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2_n_pub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Published signatures in M14 proliferation check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_pub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2_n_Ak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size-matched random signatures in M14 proliferation check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">720</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_Ak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2_raw_P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fisher P before proliferation adjustment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4e-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">raw_fisher_P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2_sep_P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mann-Whitney P, subtype separation by proliferation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MWU_P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3_min_n_per_k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum random signatures per k shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FigS3_m8_rate_by_k_observed.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min n (k &lt;= 12, n &gt;= 20)</t>
   </si>
   <si>
     <t xml:space="preserve">corp_dedup</t>
@@ -3050,9 +3158,6 @@
     <t xml:space="preserve">1,480</t>
   </si>
   <si>
-    <t xml:space="preserve">M7 n_null</t>
-  </si>
-  <si>
     <t xml:space="preserve">n_null_M14</t>
   </si>
   <si>
@@ -3060,9 +3165,6 @@
   </si>
   <si>
     <t xml:space="preserve">3,585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M14 n_null</t>
   </si>
   <si>
     <t xml:space="preserve">n_fig3_Inputmatchedrandom</t>
@@ -9867,152 +9969,152 @@
         <v>898</v>
       </c>
       <c r="B249" t="s">
+        <v>468</v>
+      </c>
+      <c r="C249" t="s">
         <v>899</v>
       </c>
-      <c r="C249" t="s">
+      <c r="D249" t="s">
         <v>900</v>
       </c>
-      <c r="D249" t="s">
+      <c r="E249" t="n">
+        <v>2375</v>
+      </c>
+      <c r="F249" t="s">
         <v>901</v>
       </c>
-      <c r="E249" t="n">
-        <v>575</v>
-      </c>
-      <c r="F249" t="s">
+      <c r="G249" t="s">
         <v>902</v>
       </c>
-      <c r="G249" t="s">
+      <c r="H249" t="s">
         <v>903</v>
-      </c>
-      <c r="H249" t="s">
-        <v>904</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
+        <v>904</v>
+      </c>
+      <c r="B250" t="s">
+        <v>468</v>
+      </c>
+      <c r="C250" t="s">
+        <v>899</v>
+      </c>
+      <c r="D250" t="s">
         <v>905</v>
       </c>
-      <c r="B250" t="s">
-        <v>899</v>
-      </c>
-      <c r="C250" t="s">
-        <v>900</v>
-      </c>
-      <c r="D250" t="s">
+      <c r="E250" t="n">
+        <v>950</v>
+      </c>
+      <c r="F250" t="s">
         <v>906</v>
       </c>
-      <c r="E250" t="n">
-        <v>473</v>
-      </c>
-      <c r="F250" t="s">
+      <c r="G250" t="s">
+        <v>902</v>
+      </c>
+      <c r="H250" t="s">
         <v>907</v>
-      </c>
-      <c r="G250" t="s">
-        <v>903</v>
-      </c>
-      <c r="H250" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="s">
+        <v>908</v>
+      </c>
+      <c r="B251" t="s">
+        <v>468</v>
+      </c>
+      <c r="C251" t="s">
+        <v>899</v>
+      </c>
+      <c r="D251" t="s">
         <v>909</v>
       </c>
-      <c r="B251" t="s">
-        <v>899</v>
-      </c>
-      <c r="C251" t="s">
-        <v>900</v>
-      </c>
-      <c r="D251" t="s">
+      <c r="E251" t="n">
+        <v>2308</v>
+      </c>
+      <c r="F251" t="s">
         <v>910</v>
       </c>
-      <c r="E251" t="n">
-        <v>281</v>
-      </c>
-      <c r="F251" t="s">
+      <c r="G251" t="s">
+        <v>902</v>
+      </c>
+      <c r="H251" t="s">
         <v>911</v>
-      </c>
-      <c r="G251" t="s">
-        <v>903</v>
-      </c>
-      <c r="H251" t="s">
-        <v>912</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="s">
+        <v>912</v>
+      </c>
+      <c r="B252" t="s">
+        <v>468</v>
+      </c>
+      <c r="C252" t="s">
         <v>913</v>
-      </c>
-      <c r="B252" t="s">
-        <v>899</v>
-      </c>
-      <c r="C252" t="s">
-        <v>900</v>
       </c>
       <c r="D252" t="s">
         <v>914</v>
       </c>
       <c r="E252" t="n">
-        <v>294</v>
+        <v>148</v>
       </c>
       <c r="F252" t="s">
+        <v>39</v>
+      </c>
+      <c r="G252" t="s">
+        <v>871</v>
+      </c>
+      <c r="H252" t="s">
         <v>915</v>
-      </c>
-      <c r="G252" t="s">
-        <v>903</v>
-      </c>
-      <c r="H252" t="s">
-        <v>916</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
+        <v>916</v>
+      </c>
+      <c r="B253" t="s">
+        <v>468</v>
+      </c>
+      <c r="C253" t="s">
+        <v>913</v>
+      </c>
+      <c r="D253" t="s">
         <v>917</v>
       </c>
-      <c r="B253" t="s">
-        <v>899</v>
-      </c>
-      <c r="C253" t="s">
-        <v>900</v>
-      </c>
-      <c r="D253" t="s">
+      <c r="E253" t="n">
+        <v>720</v>
+      </c>
+      <c r="F253" t="s">
         <v>918</v>
       </c>
-      <c r="E253" t="n">
-        <v>260</v>
-      </c>
-      <c r="F253" t="s">
+      <c r="G253" t="s">
+        <v>871</v>
+      </c>
+      <c r="H253" t="s">
         <v>919</v>
-      </c>
-      <c r="G253" t="s">
-        <v>903</v>
-      </c>
-      <c r="H253" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
+        <v>920</v>
+      </c>
+      <c r="B254" t="s">
+        <v>468</v>
+      </c>
+      <c r="C254" t="s">
+        <v>869</v>
+      </c>
+      <c r="D254" t="s">
         <v>921</v>
       </c>
-      <c r="B254" t="s">
-        <v>899</v>
-      </c>
-      <c r="C254" t="s">
-        <v>900</v>
-      </c>
-      <c r="D254" t="s">
+      <c r="E254" t="n">
+        <v>0.000000013890692</v>
+      </c>
+      <c r="F254" t="s">
         <v>922</v>
       </c>
-      <c r="E254" t="n">
-        <v>12</v>
-      </c>
-      <c r="F254" t="s">
-        <v>611</v>
-      </c>
       <c r="G254" t="s">
-        <v>903</v>
+        <v>871</v>
       </c>
       <c r="H254" t="s">
         <v>923</v>
@@ -10023,804 +10125,1012 @@
         <v>924</v>
       </c>
       <c r="B255" t="s">
-        <v>899</v>
+        <v>468</v>
       </c>
       <c r="C255" t="s">
-        <v>900</v>
+        <v>925</v>
       </c>
       <c r="D255" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="E255" t="n">
-        <v>248</v>
+        <v>0.0000000000000031086245</v>
       </c>
       <c r="F255" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="G255" t="s">
-        <v>903</v>
+        <v>871</v>
       </c>
       <c r="H255" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B256" t="s">
-        <v>899</v>
+        <v>468</v>
       </c>
       <c r="C256" t="s">
-        <v>900</v>
+        <v>930</v>
       </c>
       <c r="D256" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="E256" t="n">
-        <v>152</v>
+        <v>21</v>
       </c>
       <c r="F256" t="s">
-        <v>930</v>
+        <v>658</v>
       </c>
       <c r="G256" t="s">
-        <v>903</v>
+        <v>932</v>
       </c>
       <c r="H256" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="B257" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C257" t="s">
-        <v>900</v>
+        <v>936</v>
       </c>
       <c r="D257" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="E257" t="n">
-        <v>149</v>
+        <v>575</v>
       </c>
       <c r="F257" t="s">
-        <v>45</v>
+        <v>938</v>
       </c>
       <c r="G257" t="s">
-        <v>903</v>
+        <v>939</v>
       </c>
       <c r="H257" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="s">
+        <v>941</v>
+      </c>
+      <c r="B258" t="s">
         <v>935</v>
       </c>
-      <c r="B258" t="s">
-        <v>899</v>
-      </c>
       <c r="C258" t="s">
-        <v>900</v>
+        <v>936</v>
       </c>
       <c r="D258" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="E258" t="n">
-        <v>87</v>
+        <v>473</v>
       </c>
       <c r="F258" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="G258" t="s">
-        <v>903</v>
+        <v>939</v>
       </c>
       <c r="H258" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="s">
+        <v>945</v>
+      </c>
+      <c r="B259" t="s">
+        <v>935</v>
+      </c>
+      <c r="C259" t="s">
+        <v>936</v>
+      </c>
+      <c r="D259" t="s">
+        <v>946</v>
+      </c>
+      <c r="E259" t="n">
+        <v>281</v>
+      </c>
+      <c r="F259" t="s">
+        <v>947</v>
+      </c>
+      <c r="G259" t="s">
         <v>939</v>
       </c>
-      <c r="B259" t="s">
-        <v>899</v>
-      </c>
-      <c r="C259" t="s">
-        <v>900</v>
-      </c>
-      <c r="D259" t="s">
-        <v>940</v>
-      </c>
-      <c r="E259" t="n">
-        <v>9</v>
-      </c>
-      <c r="F259" t="s">
-        <v>941</v>
-      </c>
-      <c r="G259" t="s">
-        <v>903</v>
-      </c>
       <c r="H259" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="B260" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C260" t="s">
-        <v>900</v>
+        <v>936</v>
       </c>
       <c r="D260" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
       <c r="E260" t="n">
-        <v>13</v>
+        <v>294</v>
       </c>
       <c r="F260" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="G260" t="s">
-        <v>903</v>
+        <v>939</v>
       </c>
       <c r="H260" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B261" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C261" t="s">
-        <v>948</v>
+        <v>936</v>
       </c>
       <c r="D261" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="E261" t="n">
-        <v>11964</v>
+        <v>260</v>
       </c>
       <c r="F261" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="G261" t="s">
-        <v>951</v>
+        <v>939</v>
       </c>
       <c r="H261" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="B262" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C262" t="s">
-        <v>948</v>
+        <v>936</v>
       </c>
       <c r="D262" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="E262" t="n">
-        <v>10651</v>
+        <v>12</v>
       </c>
       <c r="F262" t="s">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="G262" t="s">
-        <v>951</v>
+        <v>939</v>
       </c>
       <c r="H262" t="s">
-        <v>104</v>
+        <v>959</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
       <c r="B263" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C263" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D263" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="E263" t="n">
-        <v>341</v>
+        <v>248</v>
       </c>
       <c r="F263" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="G263" t="s">
-        <v>959</v>
+        <v>939</v>
       </c>
       <c r="H263" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="B264" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C264" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D264" t="s">
-        <v>962</v>
+        <v>965</v>
       </c>
       <c r="E264" t="n">
-        <v>219</v>
+        <v>152</v>
       </c>
       <c r="F264" t="s">
-        <v>963</v>
+        <v>966</v>
       </c>
       <c r="G264" t="s">
-        <v>959</v>
+        <v>939</v>
       </c>
       <c r="H264" t="s">
-        <v>960</v>
+        <v>967</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="B265" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C265" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D265" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="E265" t="n">
-        <v>203</v>
+        <v>149</v>
       </c>
       <c r="F265" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G265" t="s">
-        <v>959</v>
+        <v>939</v>
       </c>
       <c r="H265" t="s">
-        <v>960</v>
+        <v>970</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="B266" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C266" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D266" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
       <c r="E266" t="n">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="F266" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="G266" t="s">
-        <v>14</v>
+        <v>939</v>
       </c>
       <c r="H266" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
       <c r="B267" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C267" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D267" t="s">
-        <v>971</v>
+        <v>976</v>
       </c>
       <c r="E267" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F267" t="s">
-        <v>972</v>
+        <v>977</v>
       </c>
       <c r="G267" t="s">
-        <v>14</v>
+        <v>939</v>
       </c>
       <c r="H267" t="s">
-        <v>969</v>
+        <v>978</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="B268" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C268" t="s">
-        <v>956</v>
+        <v>936</v>
       </c>
       <c r="D268" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="E268" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F268" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
       <c r="G268" t="s">
-        <v>14</v>
+        <v>939</v>
       </c>
       <c r="H268" t="s">
-        <v>969</v>
+        <v>982</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>976</v>
+        <v>983</v>
       </c>
       <c r="B269" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C269" t="s">
-        <v>977</v>
+        <v>984</v>
       </c>
       <c r="D269" t="s">
-        <v>978</v>
+        <v>985</v>
       </c>
       <c r="E269" t="n">
-        <v>5</v>
+        <v>11964</v>
       </c>
       <c r="F269" t="s">
-        <v>663</v>
+        <v>986</v>
       </c>
       <c r="G269" t="s">
-        <v>979</v>
+        <v>987</v>
       </c>
       <c r="H269" t="s">
-        <v>980</v>
+        <v>988</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>981</v>
+        <v>989</v>
       </c>
       <c r="B270" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C270" t="s">
-        <v>977</v>
+        <v>984</v>
       </c>
       <c r="D270" t="s">
-        <v>982</v>
+        <v>990</v>
       </c>
       <c r="E270" t="n">
-        <v>24</v>
+        <v>10651</v>
       </c>
       <c r="F270" t="s">
-        <v>983</v>
+        <v>103</v>
       </c>
       <c r="G270" t="s">
-        <v>979</v>
+        <v>987</v>
       </c>
       <c r="H270" t="s">
-        <v>984</v>
+        <v>104</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="B271" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C271" t="s">
-        <v>977</v>
+        <v>992</v>
       </c>
       <c r="D271" t="s">
-        <v>986</v>
+        <v>993</v>
       </c>
       <c r="E271" t="n">
-        <v>95</v>
+        <v>341</v>
       </c>
       <c r="F271" t="s">
-        <v>987</v>
+        <v>994</v>
       </c>
       <c r="G271" t="s">
-        <v>979</v>
+        <v>995</v>
       </c>
       <c r="H271" t="s">
-        <v>988</v>
+        <v>996</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>989</v>
+        <v>997</v>
       </c>
       <c r="B272" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C272" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D272" t="s">
-        <v>991</v>
+        <v>998</v>
       </c>
       <c r="E272" t="n">
-        <v>25</v>
+        <v>219</v>
       </c>
       <c r="F272" t="s">
-        <v>992</v>
+        <v>999</v>
       </c>
       <c r="G272" t="s">
-        <v>318</v>
+        <v>995</v>
       </c>
       <c r="H272" t="s">
-        <v>993</v>
+        <v>996</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="B273" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C273" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D273" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E273" t="n">
+        <v>203</v>
+      </c>
+      <c r="F273" t="s">
+        <v>28</v>
+      </c>
+      <c r="G273" t="s">
         <v>995</v>
       </c>
-      <c r="E273" t="n">
-        <v>10</v>
-      </c>
-      <c r="F273" t="s">
-        <v>78</v>
-      </c>
-      <c r="G273" t="s">
-        <v>318</v>
-      </c>
       <c r="H273" t="s">
-        <v>993</v>
+        <v>996</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="B274" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C274" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
       <c r="D274" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="E274" t="n">
-        <v>298</v>
+        <v>24</v>
       </c>
       <c r="F274" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="G274" t="s">
-        <v>1000</v>
+        <v>14</v>
       </c>
       <c r="H274" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="B275" t="s">
-        <v>899</v>
+        <v>935</v>
       </c>
       <c r="C275" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
       <c r="D275" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="E275" t="n">
-        <v>191</v>
+        <v>2</v>
       </c>
       <c r="F275" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="G275" t="s">
-        <v>1000</v>
+        <v>14</v>
       </c>
       <c r="H275" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B276" t="s">
+        <v>935</v>
+      </c>
+      <c r="C276" t="s">
+        <v>992</v>
+      </c>
+      <c r="D276" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" t="s">
+        <v>1011</v>
+      </c>
+      <c r="G276" t="s">
+        <v>14</v>
+      </c>
+      <c r="H276" t="s">
         <v>1005</v>
-      </c>
-      <c r="B276" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C276" t="s">
-        <v>315</v>
-      </c>
-      <c r="D276" t="s">
-        <v>1007</v>
-      </c>
-      <c r="E276" t="n">
-        <v>3700</v>
-      </c>
-      <c r="F276" t="s">
-        <v>668</v>
-      </c>
-      <c r="G276" t="s">
-        <v>318</v>
-      </c>
-      <c r="H276" t="s">
-        <v>1008</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>1009</v>
+        <v>1012</v>
       </c>
       <c r="B277" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C277" t="s">
-        <v>315</v>
+        <v>1013</v>
       </c>
       <c r="D277" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="E277" t="n">
-        <v>1480</v>
+        <v>5</v>
       </c>
       <c r="F277" t="s">
-        <v>1011</v>
+        <v>663</v>
       </c>
       <c r="G277" t="s">
-        <v>318</v>
+        <v>1015</v>
       </c>
       <c r="H277" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B278" t="s">
+        <v>935</v>
+      </c>
+      <c r="C278" t="s">
         <v>1013</v>
       </c>
-      <c r="B278" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C278" t="s">
-        <v>315</v>
-      </c>
       <c r="D278" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="E278" t="n">
-        <v>3585</v>
+        <v>24</v>
       </c>
       <c r="F278" t="s">
+        <v>1019</v>
+      </c>
+      <c r="G278" t="s">
         <v>1015</v>
       </c>
-      <c r="G278" t="s">
-        <v>318</v>
-      </c>
       <c r="H278" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="B279" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C279" t="s">
-        <v>1018</v>
+        <v>1013</v>
       </c>
       <c r="D279" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="E279" t="n">
-        <v>3700</v>
+        <v>95</v>
       </c>
       <c r="F279" t="s">
-        <v>668</v>
+        <v>1023</v>
       </c>
       <c r="G279" t="s">
-        <v>1020</v>
+        <v>1015</v>
       </c>
       <c r="H279" t="s">
-        <v>1021</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>1022</v>
+        <v>1025</v>
       </c>
       <c r="B280" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C280" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
       <c r="D280" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="E280" t="n">
-        <v>148</v>
+        <v>25</v>
       </c>
       <c r="F280" t="s">
-        <v>39</v>
+        <v>1028</v>
       </c>
       <c r="G280" t="s">
-        <v>1020</v>
+        <v>318</v>
       </c>
       <c r="H280" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
       <c r="B281" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C281" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
       <c r="D281" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="E281" t="n">
-        <v>3700</v>
+        <v>10</v>
       </c>
       <c r="F281" t="s">
-        <v>668</v>
+        <v>78</v>
       </c>
       <c r="G281" t="s">
-        <v>1020</v>
+        <v>318</v>
       </c>
       <c r="H281" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="B282" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C282" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="D282" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="E282" t="n">
-        <v>148</v>
+        <v>298</v>
       </c>
       <c r="F282" t="s">
-        <v>39</v>
+        <v>1035</v>
       </c>
       <c r="G282" t="s">
-        <v>1029</v>
+        <v>1036</v>
       </c>
       <c r="H282" t="s">
-        <v>1030</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>1031</v>
+        <v>1038</v>
       </c>
       <c r="B283" t="s">
-        <v>1006</v>
+        <v>935</v>
       </c>
       <c r="C283" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="D283" t="s">
-        <v>1032</v>
+        <v>1039</v>
       </c>
       <c r="E283" t="n">
-        <v>148</v>
+        <v>191</v>
       </c>
       <c r="F283" t="s">
-        <v>39</v>
+        <v>1040</v>
       </c>
       <c r="G283" t="s">
-        <v>1029</v>
+        <v>1036</v>
       </c>
       <c r="H283" t="s">
-        <v>1030</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>1033</v>
+        <v>1041</v>
       </c>
       <c r="B284" t="s">
-        <v>1006</v>
+        <v>1042</v>
       </c>
       <c r="C284" t="s">
-        <v>738</v>
+        <v>315</v>
       </c>
       <c r="D284" t="s">
-        <v>1034</v>
+        <v>1043</v>
       </c>
       <c r="E284" t="n">
-        <v>29600</v>
+        <v>3700</v>
       </c>
       <c r="F284" t="s">
-        <v>1035</v>
+        <v>668</v>
       </c>
       <c r="G284" t="s">
-        <v>761</v>
+        <v>318</v>
       </c>
       <c r="H284" t="s">
-        <v>15</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>1036</v>
+        <v>1045</v>
       </c>
       <c r="B285" t="s">
-        <v>1006</v>
+        <v>1042</v>
       </c>
       <c r="C285" t="s">
+        <v>315</v>
+      </c>
+      <c r="D285" t="s">
+        <v>1046</v>
+      </c>
+      <c r="E285" t="n">
+        <v>1480</v>
+      </c>
+      <c r="F285" t="s">
+        <v>1047</v>
+      </c>
+      <c r="G285" t="s">
+        <v>318</v>
+      </c>
+      <c r="H285" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B286" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C286" t="s">
+        <v>315</v>
+      </c>
+      <c r="D286" t="s">
+        <v>1049</v>
+      </c>
+      <c r="E286" t="n">
+        <v>3585</v>
+      </c>
+      <c r="F286" t="s">
+        <v>1050</v>
+      </c>
+      <c r="G286" t="s">
+        <v>318</v>
+      </c>
+      <c r="H286" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B287" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C287" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D287" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E287" t="n">
+        <v>3700</v>
+      </c>
+      <c r="F287" t="s">
+        <v>668</v>
+      </c>
+      <c r="G287" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H287" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B288" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C288" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D288" t="s">
+        <v>1057</v>
+      </c>
+      <c r="E288" t="n">
+        <v>148</v>
+      </c>
+      <c r="F288" t="s">
+        <v>39</v>
+      </c>
+      <c r="G288" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H288" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B289" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C289" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D289" t="s">
+        <v>1059</v>
+      </c>
+      <c r="E289" t="n">
+        <v>3700</v>
+      </c>
+      <c r="F289" t="s">
+        <v>668</v>
+      </c>
+      <c r="G289" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H289" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B290" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D290" t="s">
+        <v>1062</v>
+      </c>
+      <c r="E290" t="n">
+        <v>148</v>
+      </c>
+      <c r="F290" t="s">
+        <v>39</v>
+      </c>
+      <c r="G290" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H290" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B291" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D291" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E291" t="n">
+        <v>148</v>
+      </c>
+      <c r="F291" t="s">
+        <v>39</v>
+      </c>
+      <c r="G291" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H291" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B292" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C292" t="s">
+        <v>738</v>
+      </c>
+      <c r="D292" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E292" t="n">
+        <v>29600</v>
+      </c>
+      <c r="F292" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G292" t="s">
+        <v>761</v>
+      </c>
+      <c r="H292" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B293" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C293" t="s">
         <v>490</v>
       </c>
-      <c r="D285" t="s">
-        <v>1037</v>
-      </c>
-      <c r="E285" t="n">
+      <c r="D293" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E293" t="n">
         <v>200</v>
       </c>
-      <c r="F285" t="s">
+      <c r="F293" t="s">
         <v>94</v>
       </c>
-      <c r="G285" t="s">
+      <c r="G293" t="s">
         <v>812</v>
       </c>
-      <c r="H285" t="s">
+      <c r="H293" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove superseded simulation inputs; make paired_tests standalone
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_S3.xlsx
+++ b/supplementary_tables/Supplementary_Table_S3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="1037">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="1043">
   <si>
     <t xml:space="preserve">Supplementary Table S3. Every quantity reported in the text and figures, with source file and extraction rule.</t>
   </si>
@@ -518,7 +518,7 @@
     <t xml:space="preserve">2.0e-16</t>
   </si>
   <si>
-    <t xml:space="preserve">P (paired Wilcoxon, N35)</t>
+    <t xml:space="preserve">P (paired Wilcoxon)</t>
   </si>
   <si>
     <t xml:space="preserve">C2_rho_prolif_pub_TCGA</t>
@@ -674,7 +674,7 @@
     <t xml:space="preserve">7.7e-07</t>
   </si>
   <si>
-    <t xml:space="preserve">P, Input-matched (paired Wilcoxon, N35)</t>
+    <t xml:space="preserve">P, Input-matched (paired Wilcoxon)</t>
   </si>
   <si>
     <t xml:space="preserve">C2_rho_prolif_In_TCGA</t>
@@ -806,7 +806,7 @@
     <t xml:space="preserve">CMH P stratified by matched set, published vs Size-matched random Base: proliferation, stroma, immune, stage, age, sex</t>
   </si>
   <si>
-    <t xml:space="preserve">P_vs_published (CMH, N35)</t>
+    <t xml:space="preserve">P_vs_published (CMH)</t>
   </si>
   <si>
     <t xml:space="preserve">C2_resid_Sizematchedrandom_oxphos</t>
@@ -1712,12 +1712,42 @@
     <t xml:space="preserve">selected, beta 0.6, FWp</t>
   </si>
   <si>
+    <t xml:space="preserve">N1_HR_b02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fig7c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulated hazard ratio per s.d.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exp(beta), beta 0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N1_HR_b04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exp(beta), beta 0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N1_HR_b06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exp(beta), beta 0.6</t>
+  </si>
+  <si>
     <t xml:space="preserve">N2_template_T0</t>
   </si>
   <si>
-    <t xml:space="preserve">Fig7c</t>
-  </si>
-  <si>
     <t xml:space="preserve">Published signatures passing, template_T0</t>
   </si>
   <si>
@@ -2249,7 +2279,7 @@
     <t xml:space="preserve">1.5e-18</t>
   </si>
   <si>
-    <t xml:space="preserve">P, Input-matched (CMH, N35)</t>
+    <t xml:space="preserve">P, Input-matched (CMH)</t>
   </si>
   <si>
     <t xml:space="preserve">C4_M8b_Inputmatchedrandom</t>
@@ -2363,7 +2393,7 @@
     <t xml:space="preserve">0.89</t>
   </si>
   <si>
-    <t xml:space="preserve">P (CMH, N35)</t>
+    <t xml:space="preserve">P (CMH)</t>
   </si>
   <si>
     <t xml:space="preserve">C4_knk_fc_rho</t>
@@ -2468,30 +2498,21 @@
     <t xml:space="preserve">C6_pub_adjHR_GSE</t>
   </si>
   <si>
-    <t xml:space="preserve">Published median adjusted HR, GSE14520</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fig7b_sim_verdict.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">published_adjHR_median_GSE</t>
+    <t xml:space="preserve">Published median adjusted HR per s.d. (exp median |log HR|), GSE14520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exp(median_abslogHR_adj), A_vs_fitsig_k real</t>
   </si>
   <si>
     <t xml:space="preserve">C6_pub_adjHR_LIRI</t>
   </si>
   <si>
-    <t xml:space="preserve">Published median adjusted HR, LIRI-JP</t>
+    <t xml:space="preserve">Published median adjusted HR per s.d. (exp median |log HR|), LIRI-JP</t>
   </si>
   <si>
     <t xml:space="preserve">1.26</t>
   </si>
   <si>
-    <t xml:space="preserve">published_adjHR_median_LIRI</t>
-  </si>
-  <si>
     <t xml:space="preserve">S1_n_same_verdict</t>
   </si>
   <si>
@@ -2567,7 +2588,7 @@
     <t xml:space="preserve">0.39</t>
   </si>
   <si>
-    <t xml:space="preserve">adj_P (CMH, N35)</t>
+    <t xml:space="preserve">adj_P (CMH)</t>
   </si>
   <si>
     <t xml:space="preserve">S4_top25_prolif</t>
@@ -2675,7 +2696,7 @@
     <t xml:space="preserve">1.3e-09</t>
   </si>
   <si>
-    <t xml:space="preserve">raw_P (CMH, N35)</t>
+    <t xml:space="preserve">raw_P (CMH)</t>
   </si>
   <si>
     <t xml:space="preserve">S2_sep_P</t>
@@ -2690,7 +2711,7 @@
     <t xml:space="preserve">2.8e-12</t>
   </si>
   <si>
-    <t xml:space="preserve">sep_P (paired Wilcoxon, N35)</t>
+    <t xml:space="preserve">sep_P (paired Wilcoxon)</t>
   </si>
   <si>
     <t xml:space="preserve">S3_min_n_per_k</t>
@@ -3120,9 +3141,6 @@
   </si>
   <si>
     <t xml:space="preserve">Simulation runs per effect size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fig7b_sim_power.tsv</t>
   </si>
 </sst>
 </file>
@@ -7663,21 +7681,21 @@
         <v>568</v>
       </c>
       <c r="E164" t="n">
-        <v>0.50675676</v>
+        <v>1.2214028</v>
       </c>
       <c r="F164" t="s">
         <v>569</v>
       </c>
       <c r="G164" t="s">
+        <v>501</v>
+      </c>
+      <c r="H164" t="s">
         <v>570</v>
-      </c>
-      <c r="H164" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B165" t="s">
         <v>497</v>
@@ -7686,24 +7704,24 @@
         <v>567</v>
       </c>
       <c r="D165" t="s">
+        <v>568</v>
+      </c>
+      <c r="E165" t="n">
+        <v>1.4918247</v>
+      </c>
+      <c r="F165" t="s">
+        <v>572</v>
+      </c>
+      <c r="G165" t="s">
+        <v>501</v>
+      </c>
+      <c r="H165" t="s">
         <v>573</v>
-      </c>
-      <c r="E165" t="n">
-        <v>0</v>
-      </c>
-      <c r="F165" t="s">
-        <v>574</v>
-      </c>
-      <c r="G165" t="s">
-        <v>570</v>
-      </c>
-      <c r="H165" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B166" t="s">
         <v>497</v>
@@ -7712,24 +7730,24 @@
         <v>567</v>
       </c>
       <c r="D166" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="E166" t="n">
-        <v>0.040540541</v>
+        <v>1.8221188</v>
       </c>
       <c r="F166" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="G166" t="s">
-        <v>570</v>
+        <v>501</v>
       </c>
       <c r="H166" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="B167" t="s">
         <v>497</v>
@@ -7738,24 +7756,24 @@
         <v>567</v>
       </c>
       <c r="D167" t="s">
+        <v>578</v>
+      </c>
+      <c r="E167" t="n">
+        <v>0.50675676</v>
+      </c>
+      <c r="F167" t="s">
+        <v>579</v>
+      </c>
+      <c r="G167" t="s">
+        <v>580</v>
+      </c>
+      <c r="H167" t="s">
         <v>581</v>
-      </c>
-      <c r="E167" t="n">
-        <v>0</v>
-      </c>
-      <c r="F167" t="s">
-        <v>574</v>
-      </c>
-      <c r="G167" t="s">
-        <v>570</v>
-      </c>
-      <c r="H167" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B168" t="s">
         <v>497</v>
@@ -7764,24 +7782,24 @@
         <v>567</v>
       </c>
       <c r="D168" t="s">
+        <v>583</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" t="s">
         <v>584</v>
       </c>
-      <c r="E168" t="n">
-        <v>0.047297297</v>
-      </c>
-      <c r="F168" t="s">
+      <c r="G168" t="s">
+        <v>580</v>
+      </c>
+      <c r="H168" t="s">
         <v>585</v>
-      </c>
-      <c r="G168" t="s">
-        <v>570</v>
-      </c>
-      <c r="H168" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B169" t="s">
         <v>497</v>
@@ -7790,24 +7808,24 @@
         <v>567</v>
       </c>
       <c r="D169" t="s">
+        <v>587</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0.040540541</v>
+      </c>
+      <c r="F169" t="s">
         <v>588</v>
       </c>
-      <c r="E169" t="n">
-        <v>0.46621622</v>
-      </c>
-      <c r="F169" t="s">
+      <c r="G169" t="s">
+        <v>580</v>
+      </c>
+      <c r="H169" t="s">
         <v>589</v>
-      </c>
-      <c r="G169" t="s">
-        <v>570</v>
-      </c>
-      <c r="H169" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B170" t="s">
         <v>497</v>
@@ -7816,24 +7834,24 @@
         <v>567</v>
       </c>
       <c r="D170" t="s">
+        <v>591</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" t="s">
+        <v>584</v>
+      </c>
+      <c r="G170" t="s">
+        <v>580</v>
+      </c>
+      <c r="H170" t="s">
         <v>592</v>
-      </c>
-      <c r="E170" t="n">
-        <v>0.047297297</v>
-      </c>
-      <c r="F170" t="s">
-        <v>585</v>
-      </c>
-      <c r="G170" t="s">
-        <v>570</v>
-      </c>
-      <c r="H170" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B171" t="s">
         <v>497</v>
@@ -7842,253 +7860,253 @@
         <v>567</v>
       </c>
       <c r="D171" t="s">
+        <v>594</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0.047297297</v>
+      </c>
+      <c r="F171" t="s">
         <v>595</v>
       </c>
-      <c r="E171" t="n">
-        <v>0.21510503</v>
-      </c>
-      <c r="F171" t="s">
+      <c r="G171" t="s">
+        <v>580</v>
+      </c>
+      <c r="H171" t="s">
         <v>596</v>
-      </c>
-      <c r="G171" t="s">
-        <v>597</v>
-      </c>
-      <c r="H171" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="s">
+        <v>597</v>
+      </c>
+      <c r="B172" t="s">
+        <v>497</v>
+      </c>
+      <c r="C172" t="s">
+        <v>567</v>
+      </c>
+      <c r="D172" t="s">
+        <v>598</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0.46621622</v>
+      </c>
+      <c r="F172" t="s">
         <v>599</v>
       </c>
-      <c r="B172" t="s">
-        <v>312</v>
-      </c>
-      <c r="C172" t="s">
+      <c r="G172" t="s">
+        <v>580</v>
+      </c>
+      <c r="H172" t="s">
         <v>600</v>
-      </c>
-      <c r="D172" t="s">
-        <v>601</v>
-      </c>
-      <c r="E172" t="n">
-        <v>145</v>
-      </c>
-      <c r="F172" t="s">
-        <v>602</v>
-      </c>
-      <c r="G172" t="s">
-        <v>603</v>
-      </c>
-      <c r="H172" t="s">
-        <v>604</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="B173" t="s">
-        <v>312</v>
+        <v>497</v>
       </c>
       <c r="C173" t="s">
-        <v>600</v>
+        <v>567</v>
       </c>
       <c r="D173" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E173" t="n">
-        <v>82</v>
+        <v>0.047297297</v>
       </c>
       <c r="F173" t="s">
-        <v>607</v>
+        <v>595</v>
       </c>
       <c r="G173" t="s">
+        <v>580</v>
+      </c>
+      <c r="H173" t="s">
         <v>603</v>
-      </c>
-      <c r="H173" t="s">
-        <v>608</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="B174" t="s">
-        <v>312</v>
+        <v>497</v>
       </c>
       <c r="C174" t="s">
-        <v>600</v>
+        <v>567</v>
       </c>
       <c r="D174" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="E174" t="n">
-        <v>6</v>
+        <v>0.21510503</v>
       </c>
       <c r="F174" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="G174" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="H174" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="B175" t="s">
         <v>312</v>
       </c>
       <c r="C175" t="s">
-        <v>600</v>
+        <v>610</v>
       </c>
       <c r="D175" t="s">
+        <v>611</v>
+      </c>
+      <c r="E175" t="n">
+        <v>145</v>
+      </c>
+      <c r="F175" t="s">
+        <v>612</v>
+      </c>
+      <c r="G175" t="s">
+        <v>613</v>
+      </c>
+      <c r="H175" t="s">
         <v>614</v>
-      </c>
-      <c r="E175" t="n">
-        <v>6</v>
-      </c>
-      <c r="F175" t="s">
-        <v>611</v>
-      </c>
-      <c r="G175" t="s">
-        <v>603</v>
-      </c>
-      <c r="H175" t="s">
-        <v>615</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B176" t="s">
         <v>312</v>
       </c>
       <c r="C176" t="s">
+        <v>610</v>
+      </c>
+      <c r="D176" t="s">
+        <v>616</v>
+      </c>
+      <c r="E176" t="n">
+        <v>82</v>
+      </c>
+      <c r="F176" t="s">
         <v>617</v>
       </c>
-      <c r="D176" t="s">
+      <c r="G176" t="s">
+        <v>613</v>
+      </c>
+      <c r="H176" t="s">
         <v>618</v>
-      </c>
-      <c r="E176" t="n">
-        <v>12</v>
-      </c>
-      <c r="F176" t="s">
-        <v>619</v>
-      </c>
-      <c r="G176" t="s">
-        <v>40</v>
-      </c>
-      <c r="H176" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B177" t="s">
         <v>312</v>
       </c>
       <c r="C177" t="s">
+        <v>610</v>
+      </c>
+      <c r="D177" t="s">
+        <v>620</v>
+      </c>
+      <c r="E177" t="n">
+        <v>6</v>
+      </c>
+      <c r="F177" t="s">
+        <v>621</v>
+      </c>
+      <c r="G177" t="s">
+        <v>613</v>
+      </c>
+      <c r="H177" t="s">
         <v>622</v>
-      </c>
-      <c r="D177" t="s">
-        <v>623</v>
-      </c>
-      <c r="E177" t="n">
-        <v>2.2115085</v>
-      </c>
-      <c r="F177" t="s">
-        <v>624</v>
-      </c>
-      <c r="G177" t="s">
-        <v>625</v>
-      </c>
-      <c r="H177" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="B178" t="s">
         <v>312</v>
       </c>
       <c r="C178" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
       <c r="D178" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="E178" t="n">
-        <v>0.0000087790673</v>
+        <v>6</v>
       </c>
       <c r="F178" t="s">
-        <v>629</v>
+        <v>621</v>
       </c>
       <c r="G178" t="s">
+        <v>613</v>
+      </c>
+      <c r="H178" t="s">
         <v>625</v>
-      </c>
-      <c r="H178" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="B179" t="s">
         <v>312</v>
       </c>
       <c r="C179" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="D179" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="E179" t="n">
-        <v>2.3001483</v>
+        <v>12</v>
       </c>
       <c r="F179" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="G179" t="s">
-        <v>625</v>
+        <v>40</v>
       </c>
       <c r="H179" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="B180" t="s">
         <v>312</v>
       </c>
       <c r="C180" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="D180" t="s">
+        <v>633</v>
+      </c>
+      <c r="E180" t="n">
+        <v>2.2115085</v>
+      </c>
+      <c r="F180" t="s">
+        <v>634</v>
+      </c>
+      <c r="G180" t="s">
         <v>635</v>
       </c>
-      <c r="E180" t="n">
-        <v>0.00015114703</v>
-      </c>
-      <c r="F180" t="s">
+      <c r="H180" t="s">
         <v>636</v>
-      </c>
-      <c r="G180" t="s">
-        <v>625</v>
-      </c>
-      <c r="H180" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="181">
@@ -8099,261 +8117,261 @@
         <v>312</v>
       </c>
       <c r="C181" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="D181" t="s">
         <v>638</v>
       </c>
       <c r="E181" t="n">
-        <v>1.8804664</v>
+        <v>0.0000087790673</v>
       </c>
       <c r="F181" t="s">
         <v>639</v>
       </c>
       <c r="G181" t="s">
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="H181" t="s">
-        <v>626</v>
+        <v>640</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B182" t="s">
         <v>312</v>
       </c>
       <c r="C182" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="D182" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E182" t="n">
-        <v>0.067061721</v>
+        <v>2.3001483</v>
       </c>
       <c r="F182" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="G182" t="s">
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="H182" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B183" t="s">
         <v>312</v>
       </c>
       <c r="C183" t="s">
-        <v>644</v>
+        <v>632</v>
       </c>
       <c r="D183" t="s">
         <v>645</v>
       </c>
       <c r="E183" t="n">
-        <v>0.7199565</v>
+        <v>0.00015114703</v>
       </c>
       <c r="F183" t="s">
         <v>646</v>
       </c>
       <c r="G183" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
       <c r="H183" t="s">
-        <v>648</v>
+        <v>640</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B184" t="s">
         <v>312</v>
       </c>
       <c r="C184" t="s">
-        <v>644</v>
+        <v>632</v>
       </c>
       <c r="D184" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="E184" t="n">
-        <v>0.70161104</v>
+        <v>1.8804664</v>
       </c>
       <c r="F184" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="G184" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
       <c r="H184" t="s">
-        <v>648</v>
+        <v>636</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B185" t="s">
         <v>312</v>
       </c>
       <c r="C185" t="s">
-        <v>644</v>
+        <v>632</v>
       </c>
       <c r="D185" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="E185" t="n">
-        <v>0.6921733</v>
+        <v>0.067061721</v>
       </c>
       <c r="F185" t="s">
-        <v>131</v>
+        <v>652</v>
       </c>
       <c r="G185" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
       <c r="H185" t="s">
-        <v>648</v>
+        <v>640</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B186" t="s">
         <v>312</v>
       </c>
       <c r="C186" t="s">
+        <v>654</v>
+      </c>
+      <c r="D186" t="s">
         <v>655</v>
       </c>
-      <c r="D186" t="s">
+      <c r="E186" t="n">
+        <v>0.7199565</v>
+      </c>
+      <c r="F186" t="s">
         <v>656</v>
       </c>
-      <c r="E186" t="n">
-        <v>1.5551027</v>
-      </c>
-      <c r="F186" t="s">
+      <c r="G186" t="s">
         <v>657</v>
       </c>
-      <c r="G186" t="s">
+      <c r="H186" t="s">
         <v>658</v>
-      </c>
-      <c r="H186" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B187" t="s">
         <v>312</v>
       </c>
       <c r="C187" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D187" t="s">
+        <v>660</v>
+      </c>
+      <c r="E187" t="n">
+        <v>0.70161104</v>
+      </c>
+      <c r="F187" t="s">
         <v>661</v>
       </c>
-      <c r="E187" t="n">
-        <v>0.0000085970058</v>
-      </c>
-      <c r="F187" t="s">
-        <v>662</v>
-      </c>
       <c r="G187" t="s">
+        <v>657</v>
+      </c>
+      <c r="H187" t="s">
         <v>658</v>
-      </c>
-      <c r="H187" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B188" t="s">
         <v>312</v>
       </c>
       <c r="C188" t="s">
-        <v>664</v>
+        <v>654</v>
       </c>
       <c r="D188" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E188" t="n">
-        <v>21</v>
+        <v>0.6921733</v>
       </c>
       <c r="F188" t="s">
-        <v>666</v>
+        <v>131</v>
       </c>
       <c r="G188" t="s">
-        <v>667</v>
+        <v>657</v>
       </c>
       <c r="H188" t="s">
-        <v>668</v>
+        <v>658</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="B189" t="s">
         <v>312</v>
       </c>
       <c r="C189" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D189" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="E189" t="n">
-        <v>5</v>
+        <v>1.5551027</v>
       </c>
       <c r="F189" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="G189" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="H189" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="B190" t="s">
         <v>312</v>
       </c>
       <c r="C190" t="s">
-        <v>674</v>
+        <v>665</v>
       </c>
       <c r="D190" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="E190" t="n">
-        <v>3700</v>
+        <v>0.0000085970058</v>
       </c>
       <c r="F190" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="G190" t="s">
-        <v>677</v>
+        <v>668</v>
       </c>
       <c r="H190" t="s">
-        <v>15</v>
+        <v>669</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="B191" t="s">
         <v>312</v>
@@ -8362,24 +8380,24 @@
         <v>674</v>
       </c>
       <c r="D191" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="E191" t="n">
-        <v>0.46432432</v>
+        <v>21</v>
       </c>
       <c r="F191" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="G191" t="s">
         <v>677</v>
       </c>
       <c r="H191" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B192" t="s">
         <v>312</v>
@@ -8388,175 +8406,175 @@
         <v>674</v>
       </c>
       <c r="D192" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="E192" t="n">
-        <v>0.9627027</v>
+        <v>5</v>
       </c>
       <c r="F192" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="G192" t="s">
         <v>677</v>
       </c>
       <c r="H192" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B193" t="s">
         <v>312</v>
       </c>
       <c r="C193" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D193" t="s">
+        <v>685</v>
+      </c>
+      <c r="E193" t="n">
+        <v>3700</v>
+      </c>
+      <c r="F193" t="s">
         <v>686</v>
       </c>
-      <c r="E193" t="n">
-        <v>0.12378378</v>
-      </c>
-      <c r="F193" t="s">
-        <v>619</v>
-      </c>
       <c r="G193" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H193" t="s">
-        <v>681</v>
+        <v>15</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B194" t="s">
         <v>312</v>
       </c>
       <c r="C194" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D194" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="E194" t="n">
-        <v>0.25810811</v>
+        <v>0.46432432</v>
       </c>
       <c r="F194" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="G194" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H194" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="B195" t="s">
         <v>312</v>
       </c>
       <c r="C195" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D195" t="s">
+        <v>693</v>
+      </c>
+      <c r="E195" t="n">
+        <v>0.9627027</v>
+      </c>
+      <c r="F195" t="s">
+        <v>694</v>
+      </c>
+      <c r="G195" t="s">
+        <v>687</v>
+      </c>
+      <c r="H195" t="s">
         <v>691</v>
-      </c>
-      <c r="E195" t="n">
-        <v>0.59351351</v>
-      </c>
-      <c r="F195" t="s">
-        <v>692</v>
-      </c>
-      <c r="G195" t="s">
-        <v>677</v>
-      </c>
-      <c r="H195" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B196" t="s">
         <v>312</v>
       </c>
       <c r="C196" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D196" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E196" t="n">
-        <v>0.17945946</v>
+        <v>0.12378378</v>
       </c>
       <c r="F196" t="s">
-        <v>695</v>
+        <v>629</v>
       </c>
       <c r="G196" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H196" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B197" t="s">
         <v>312</v>
       </c>
       <c r="C197" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D197" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="E197" t="n">
-        <v>0.3127027</v>
+        <v>0.25810811</v>
       </c>
       <c r="F197" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G197" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H197" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B198" t="s">
         <v>312</v>
       </c>
       <c r="C198" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D198" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E198" t="n">
-        <v>2.2507465</v>
+        <v>0.59351351</v>
       </c>
       <c r="F198" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="G198" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H198" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
     </row>
     <row r="199">
@@ -8567,22 +8585,22 @@
         <v>312</v>
       </c>
       <c r="C199" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D199" t="s">
         <v>704</v>
       </c>
       <c r="E199" t="n">
-        <v>1.5952292</v>
+        <v>0.17945946</v>
       </c>
       <c r="F199" t="s">
         <v>705</v>
       </c>
       <c r="G199" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H199" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
     </row>
     <row r="200">
@@ -8593,22 +8611,22 @@
         <v>312</v>
       </c>
       <c r="C200" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D200" t="s">
         <v>707</v>
       </c>
       <c r="E200" t="n">
-        <v>3.1170571</v>
+        <v>0.3127027</v>
       </c>
       <c r="F200" t="s">
         <v>708</v>
       </c>
       <c r="G200" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H200" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
     </row>
     <row r="201">
@@ -8619,48 +8637,48 @@
         <v>312</v>
       </c>
       <c r="C201" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D201" t="s">
         <v>710</v>
       </c>
       <c r="E201" t="n">
-        <v>1.6332443</v>
+        <v>2.2507465</v>
       </c>
       <c r="F201" t="s">
         <v>711</v>
       </c>
       <c r="G201" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H201" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B202" t="s">
         <v>312</v>
       </c>
       <c r="C202" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D202" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E202" t="n">
-        <v>0.9827027</v>
+        <v>1.5952292</v>
       </c>
       <c r="F202" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="G202" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H202" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="203">
@@ -8671,22 +8689,22 @@
         <v>312</v>
       </c>
       <c r="C203" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D203" t="s">
         <v>717</v>
       </c>
       <c r="E203" t="n">
-        <v>0.51567568</v>
+        <v>3.1170571</v>
       </c>
       <c r="F203" t="s">
         <v>718</v>
       </c>
       <c r="G203" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H203" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="204">
@@ -8697,22 +8715,22 @@
         <v>312</v>
       </c>
       <c r="C204" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D204" t="s">
         <v>720</v>
       </c>
       <c r="E204" t="n">
-        <v>0.51513514</v>
+        <v>1.6332443</v>
       </c>
       <c r="F204" t="s">
         <v>721</v>
       </c>
       <c r="G204" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H204" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="205">
@@ -8723,178 +8741,178 @@
         <v>312</v>
       </c>
       <c r="C205" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D205" t="s">
         <v>723</v>
       </c>
       <c r="E205" t="n">
-        <v>0.98432432</v>
+        <v>0.9827027</v>
       </c>
       <c r="F205" t="s">
         <v>724</v>
       </c>
       <c r="G205" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="H205" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="s">
+        <v>726</v>
+      </c>
+      <c r="B206" t="s">
+        <v>312</v>
+      </c>
+      <c r="C206" t="s">
+        <v>684</v>
+      </c>
+      <c r="D206" t="s">
+        <v>727</v>
+      </c>
+      <c r="E206" t="n">
+        <v>0.51567568</v>
+      </c>
+      <c r="F206" t="s">
+        <v>728</v>
+      </c>
+      <c r="G206" t="s">
+        <v>687</v>
+      </c>
+      <c r="H206" t="s">
         <v>725</v>
-      </c>
-      <c r="B206" t="s">
-        <v>726</v>
-      </c>
-      <c r="C206" t="s">
-        <v>727</v>
-      </c>
-      <c r="D206" t="s">
-        <v>728</v>
-      </c>
-      <c r="E206" t="n">
-        <v>0.87162162</v>
-      </c>
-      <c r="F206" t="s">
-        <v>400</v>
-      </c>
-      <c r="G206" t="s">
-        <v>729</v>
-      </c>
-      <c r="H206" t="s">
-        <v>730</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="s">
+        <v>729</v>
+      </c>
+      <c r="B207" t="s">
+        <v>312</v>
+      </c>
+      <c r="C207" t="s">
+        <v>684</v>
+      </c>
+      <c r="D207" t="s">
+        <v>730</v>
+      </c>
+      <c r="E207" t="n">
+        <v>0.51513514</v>
+      </c>
+      <c r="F207" t="s">
         <v>731</v>
       </c>
-      <c r="B207" t="s">
-        <v>726</v>
-      </c>
-      <c r="C207" t="s">
-        <v>727</v>
-      </c>
-      <c r="D207" t="s">
-        <v>732</v>
-      </c>
-      <c r="E207" t="n">
-        <v>0.9527027</v>
-      </c>
-      <c r="F207" t="s">
-        <v>374</v>
-      </c>
       <c r="G207" t="s">
-        <v>729</v>
+        <v>687</v>
       </c>
       <c r="H207" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="s">
+        <v>732</v>
+      </c>
+      <c r="B208" t="s">
+        <v>312</v>
+      </c>
+      <c r="C208" t="s">
+        <v>684</v>
+      </c>
+      <c r="D208" t="s">
         <v>733</v>
       </c>
-      <c r="B208" t="s">
-        <v>726</v>
-      </c>
-      <c r="C208" t="s">
-        <v>727</v>
-      </c>
-      <c r="D208" t="s">
+      <c r="E208" t="n">
+        <v>0.98432432</v>
+      </c>
+      <c r="F208" t="s">
         <v>734</v>
       </c>
-      <c r="E208" t="n">
-        <v>0.76459459</v>
-      </c>
-      <c r="F208" t="s">
-        <v>735</v>
-      </c>
       <c r="G208" t="s">
-        <v>729</v>
+        <v>687</v>
       </c>
       <c r="H208" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="s">
+        <v>735</v>
+      </c>
+      <c r="B209" t="s">
         <v>736</v>
       </c>
-      <c r="B209" t="s">
-        <v>726</v>
-      </c>
       <c r="C209" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="D209" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E209" t="n">
-        <v>0.9672973</v>
+        <v>0.87162162</v>
       </c>
       <c r="F209" t="s">
-        <v>738</v>
+        <v>400</v>
       </c>
       <c r="G209" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="H209" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="s">
+        <v>741</v>
+      </c>
+      <c r="B210" t="s">
+        <v>736</v>
+      </c>
+      <c r="C210" t="s">
+        <v>737</v>
+      </c>
+      <c r="D210" t="s">
+        <v>742</v>
+      </c>
+      <c r="E210" t="n">
+        <v>0.9527027</v>
+      </c>
+      <c r="F210" t="s">
+        <v>374</v>
+      </c>
+      <c r="G210" t="s">
         <v>739</v>
       </c>
-      <c r="B210" t="s">
-        <v>726</v>
-      </c>
-      <c r="C210" t="s">
-        <v>727</v>
-      </c>
-      <c r="D210" t="s">
+      <c r="H210" t="s">
         <v>740</v>
-      </c>
-      <c r="E210" t="n">
-        <v>0.50378378</v>
-      </c>
-      <c r="F210" t="s">
-        <v>741</v>
-      </c>
-      <c r="G210" t="s">
-        <v>729</v>
-      </c>
-      <c r="H210" t="s">
-        <v>730</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B211" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C211" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="D211" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E211" t="n">
-        <v>0.000000000000000001497867</v>
+        <v>0.76459459</v>
       </c>
       <c r="F211" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="G211" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="H211" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
     </row>
     <row r="212">
@@ -8902,25 +8920,25 @@
         <v>746</v>
       </c>
       <c r="B212" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C212" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="D212" t="s">
         <v>747</v>
       </c>
       <c r="E212" t="n">
-        <v>0.68513514</v>
+        <v>0.9672973</v>
       </c>
       <c r="F212" t="s">
         <v>748</v>
       </c>
       <c r="G212" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="H212" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
     </row>
     <row r="213">
@@ -8928,25 +8946,25 @@
         <v>749</v>
       </c>
       <c r="B213" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C213" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="D213" t="s">
         <v>750</v>
       </c>
       <c r="E213" t="n">
-        <v>0.0000000000053734416</v>
+        <v>0.50378378</v>
       </c>
       <c r="F213" t="s">
         <v>751</v>
       </c>
       <c r="G213" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="H213" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
     </row>
     <row r="214">
@@ -8954,204 +8972,204 @@
         <v>752</v>
       </c>
       <c r="B214" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C214" t="s">
+        <v>737</v>
+      </c>
+      <c r="D214" t="s">
         <v>753</v>
       </c>
-      <c r="D214" t="s">
+      <c r="E214" t="n">
+        <v>0.000000000000000001497867</v>
+      </c>
+      <c r="F214" t="s">
         <v>754</v>
       </c>
-      <c r="E214" t="n">
-        <v>83</v>
-      </c>
-      <c r="F214" t="s">
+      <c r="G214" t="s">
+        <v>739</v>
+      </c>
+      <c r="H214" t="s">
         <v>755</v>
-      </c>
-      <c r="G214" t="s">
-        <v>756</v>
-      </c>
-      <c r="H214" t="s">
-        <v>757</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="s">
+        <v>756</v>
+      </c>
+      <c r="B215" t="s">
+        <v>736</v>
+      </c>
+      <c r="C215" t="s">
+        <v>737</v>
+      </c>
+      <c r="D215" t="s">
+        <v>757</v>
+      </c>
+      <c r="E215" t="n">
+        <v>0.68513514</v>
+      </c>
+      <c r="F215" t="s">
         <v>758</v>
       </c>
-      <c r="B215" t="s">
-        <v>726</v>
-      </c>
-      <c r="C215" t="s">
-        <v>753</v>
-      </c>
-      <c r="D215" t="s">
-        <v>759</v>
-      </c>
-      <c r="E215" t="n">
-        <v>0.85542169</v>
-      </c>
-      <c r="F215" t="s">
-        <v>760</v>
-      </c>
       <c r="G215" t="s">
-        <v>756</v>
+        <v>739</v>
       </c>
       <c r="H215" t="s">
-        <v>761</v>
+        <v>740</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B216" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C216" t="s">
-        <v>753</v>
+        <v>737</v>
       </c>
       <c r="D216" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="E216" t="n">
-        <v>6</v>
+        <v>0.0000000000053734416</v>
       </c>
       <c r="F216" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="G216" t="s">
-        <v>756</v>
+        <v>739</v>
       </c>
       <c r="H216" t="s">
-        <v>765</v>
+        <v>755</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="s">
+        <v>762</v>
+      </c>
+      <c r="B217" t="s">
+        <v>736</v>
+      </c>
+      <c r="C217" t="s">
+        <v>763</v>
+      </c>
+      <c r="D217" t="s">
+        <v>764</v>
+      </c>
+      <c r="E217" t="n">
+        <v>83</v>
+      </c>
+      <c r="F217" t="s">
+        <v>765</v>
+      </c>
+      <c r="G217" t="s">
         <v>766</v>
       </c>
-      <c r="B217" t="s">
-        <v>726</v>
-      </c>
-      <c r="C217" t="s">
-        <v>753</v>
-      </c>
-      <c r="D217" t="s">
+      <c r="H217" t="s">
         <v>767</v>
-      </c>
-      <c r="E217" t="n">
-        <v>860</v>
-      </c>
-      <c r="F217" t="s">
-        <v>768</v>
-      </c>
-      <c r="G217" t="s">
-        <v>769</v>
-      </c>
-      <c r="H217" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="s">
+        <v>768</v>
+      </c>
+      <c r="B218" t="s">
+        <v>736</v>
+      </c>
+      <c r="C218" t="s">
+        <v>763</v>
+      </c>
+      <c r="D218" t="s">
+        <v>769</v>
+      </c>
+      <c r="E218" t="n">
+        <v>0.85542169</v>
+      </c>
+      <c r="F218" t="s">
+        <v>770</v>
+      </c>
+      <c r="G218" t="s">
+        <v>766</v>
+      </c>
+      <c r="H218" t="s">
         <v>771</v>
-      </c>
-      <c r="B218" t="s">
-        <v>726</v>
-      </c>
-      <c r="C218" t="s">
-        <v>753</v>
-      </c>
-      <c r="D218" t="s">
-        <v>772</v>
-      </c>
-      <c r="E218" t="n">
-        <v>35</v>
-      </c>
-      <c r="F218" t="s">
-        <v>31</v>
-      </c>
-      <c r="G218" t="s">
-        <v>769</v>
-      </c>
-      <c r="H218" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="s">
+        <v>772</v>
+      </c>
+      <c r="B219" t="s">
+        <v>736</v>
+      </c>
+      <c r="C219" t="s">
+        <v>763</v>
+      </c>
+      <c r="D219" t="s">
+        <v>773</v>
+      </c>
+      <c r="E219" t="n">
+        <v>6</v>
+      </c>
+      <c r="F219" t="s">
         <v>774</v>
       </c>
-      <c r="B219" t="s">
-        <v>726</v>
-      </c>
-      <c r="C219" t="s">
-        <v>753</v>
-      </c>
-      <c r="D219" t="s">
+      <c r="G219" t="s">
+        <v>766</v>
+      </c>
+      <c r="H219" t="s">
         <v>775</v>
-      </c>
-      <c r="E219" t="n">
-        <v>0.047297297</v>
-      </c>
-      <c r="F219" t="s">
-        <v>443</v>
-      </c>
-      <c r="G219" t="s">
-        <v>776</v>
-      </c>
-      <c r="H219" t="s">
-        <v>730</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="s">
+        <v>776</v>
+      </c>
+      <c r="B220" t="s">
+        <v>736</v>
+      </c>
+      <c r="C220" t="s">
+        <v>763</v>
+      </c>
+      <c r="D220" t="s">
         <v>777</v>
       </c>
-      <c r="B220" t="s">
-        <v>726</v>
-      </c>
-      <c r="C220" t="s">
-        <v>753</v>
-      </c>
-      <c r="D220" t="s">
+      <c r="E220" t="n">
+        <v>860</v>
+      </c>
+      <c r="F220" t="s">
         <v>778</v>
       </c>
-      <c r="E220" t="n">
-        <v>0.049594595</v>
-      </c>
-      <c r="F220" t="s">
+      <c r="G220" t="s">
         <v>779</v>
       </c>
-      <c r="G220" t="s">
-        <v>776</v>
-      </c>
       <c r="H220" t="s">
-        <v>730</v>
+        <v>780</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="B221" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C221" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="D221" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="E221" t="n">
-        <v>0.89448562</v>
+        <v>35</v>
       </c>
       <c r="F221" t="s">
-        <v>782</v>
+        <v>31</v>
       </c>
       <c r="G221" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="H221" t="s">
         <v>783</v>
@@ -9162,126 +9180,126 @@
         <v>784</v>
       </c>
       <c r="B222" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="C222" t="s">
+        <v>763</v>
+      </c>
+      <c r="D222" t="s">
         <v>785</v>
       </c>
-      <c r="D222" t="s">
+      <c r="E222" t="n">
+        <v>0.047297297</v>
+      </c>
+      <c r="F222" t="s">
+        <v>443</v>
+      </c>
+      <c r="G222" t="s">
         <v>786</v>
       </c>
-      <c r="E222" t="n">
-        <v>0.9932</v>
-      </c>
-      <c r="F222" t="s">
-        <v>787</v>
-      </c>
-      <c r="G222" t="s">
-        <v>788</v>
-      </c>
       <c r="H222" t="s">
-        <v>789</v>
+        <v>740</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="B223" t="s">
-        <v>791</v>
+        <v>736</v>
       </c>
       <c r="C223" t="s">
-        <v>792</v>
+        <v>763</v>
       </c>
       <c r="D223" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="E223" t="n">
-        <v>0.60810811</v>
+        <v>0.049594595</v>
       </c>
       <c r="F223" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="G223" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="H223" t="s">
-        <v>256</v>
+        <v>740</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>796</v>
+        <v>790</v>
       </c>
       <c r="B224" t="s">
+        <v>736</v>
+      </c>
+      <c r="C224" t="s">
+        <v>763</v>
+      </c>
+      <c r="D224" t="s">
         <v>791</v>
       </c>
-      <c r="C224" t="s">
+      <c r="E224" t="n">
+        <v>0.89448562</v>
+      </c>
+      <c r="F224" t="s">
         <v>792</v>
       </c>
-      <c r="D224" t="s">
-        <v>797</v>
-      </c>
-      <c r="E224" t="n">
-        <v>0.35540541</v>
-      </c>
-      <c r="F224" t="s">
-        <v>798</v>
-      </c>
       <c r="G224" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="H224" t="s">
-        <v>256</v>
+        <v>793</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="s">
+        <v>794</v>
+      </c>
+      <c r="B225" t="s">
+        <v>736</v>
+      </c>
+      <c r="C225" t="s">
+        <v>795</v>
+      </c>
+      <c r="D225" t="s">
+        <v>796</v>
+      </c>
+      <c r="E225" t="n">
+        <v>0.9932</v>
+      </c>
+      <c r="F225" t="s">
+        <v>797</v>
+      </c>
+      <c r="G225" t="s">
+        <v>798</v>
+      </c>
+      <c r="H225" t="s">
         <v>799</v>
-      </c>
-      <c r="B225" t="s">
-        <v>791</v>
-      </c>
-      <c r="C225" t="s">
-        <v>792</v>
-      </c>
-      <c r="D225" t="s">
-        <v>800</v>
-      </c>
-      <c r="E225" t="n">
-        <v>0.0000000001457713</v>
-      </c>
-      <c r="F225" t="s">
-        <v>801</v>
-      </c>
-      <c r="G225" t="s">
-        <v>795</v>
-      </c>
-      <c r="H225" t="s">
-        <v>783</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="s">
+        <v>800</v>
+      </c>
+      <c r="B226" t="s">
+        <v>801</v>
+      </c>
+      <c r="C226" t="s">
         <v>802</v>
-      </c>
-      <c r="B226" t="s">
-        <v>791</v>
-      </c>
-      <c r="C226" t="s">
-        <v>792</v>
       </c>
       <c r="D226" t="s">
         <v>803</v>
       </c>
       <c r="E226" t="n">
-        <v>0.45162162</v>
+        <v>0.60810811</v>
       </c>
       <c r="F226" t="s">
         <v>804</v>
       </c>
       <c r="G226" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
       <c r="H226" t="s">
         <v>256</v>
@@ -9289,1446 +9307,1446 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
+        <v>806</v>
+      </c>
+      <c r="B227" t="s">
+        <v>801</v>
+      </c>
+      <c r="C227" t="s">
+        <v>802</v>
+      </c>
+      <c r="D227" t="s">
+        <v>807</v>
+      </c>
+      <c r="E227" t="n">
+        <v>0.35540541</v>
+      </c>
+      <c r="F227" t="s">
+        <v>808</v>
+      </c>
+      <c r="G227" t="s">
         <v>805</v>
       </c>
-      <c r="B227" t="s">
-        <v>791</v>
-      </c>
-      <c r="C227" t="s">
-        <v>792</v>
-      </c>
-      <c r="D227" t="s">
-        <v>806</v>
-      </c>
-      <c r="E227" t="n">
-        <v>0.000073088331</v>
-      </c>
-      <c r="F227" t="s">
-        <v>807</v>
-      </c>
-      <c r="G227" t="s">
-        <v>795</v>
-      </c>
       <c r="H227" t="s">
-        <v>783</v>
+        <v>256</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B228" t="s">
-        <v>791</v>
+        <v>801</v>
       </c>
       <c r="C228" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="D228" t="s">
         <v>810</v>
       </c>
       <c r="E228" t="n">
-        <v>23.215385</v>
+        <v>0.0000000001457713</v>
       </c>
       <c r="F228" t="s">
         <v>811</v>
       </c>
       <c r="G228" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="H228" t="s">
-        <v>813</v>
+        <v>793</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="s">
+        <v>812</v>
+      </c>
+      <c r="B229" t="s">
+        <v>801</v>
+      </c>
+      <c r="C229" t="s">
+        <v>802</v>
+      </c>
+      <c r="D229" t="s">
+        <v>813</v>
+      </c>
+      <c r="E229" t="n">
+        <v>0.45162162</v>
+      </c>
+      <c r="F229" t="s">
         <v>814</v>
       </c>
-      <c r="B229" t="s">
-        <v>791</v>
-      </c>
-      <c r="C229" t="s">
-        <v>809</v>
-      </c>
-      <c r="D229" t="s">
-        <v>815</v>
-      </c>
-      <c r="E229" t="n">
-        <v>8</v>
-      </c>
-      <c r="F229" t="s">
-        <v>117</v>
-      </c>
       <c r="G229" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="H229" t="s">
-        <v>816</v>
+        <v>256</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="s">
+        <v>815</v>
+      </c>
+      <c r="B230" t="s">
+        <v>801</v>
+      </c>
+      <c r="C230" t="s">
+        <v>802</v>
+      </c>
+      <c r="D230" t="s">
+        <v>816</v>
+      </c>
+      <c r="E230" t="n">
+        <v>0.000073088331</v>
+      </c>
+      <c r="F230" t="s">
         <v>817</v>
       </c>
-      <c r="B230" t="s">
-        <v>497</v>
-      </c>
-      <c r="C230" t="s">
-        <v>498</v>
-      </c>
-      <c r="D230" t="s">
-        <v>818</v>
-      </c>
-      <c r="E230" t="n">
-        <v>1.2232249</v>
-      </c>
-      <c r="F230" t="s">
-        <v>819</v>
-      </c>
       <c r="G230" t="s">
-        <v>820</v>
+        <v>805</v>
       </c>
       <c r="H230" t="s">
-        <v>821</v>
+        <v>793</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="s">
+        <v>818</v>
+      </c>
+      <c r="B231" t="s">
+        <v>801</v>
+      </c>
+      <c r="C231" t="s">
+        <v>819</v>
+      </c>
+      <c r="D231" t="s">
+        <v>820</v>
+      </c>
+      <c r="E231" t="n">
+        <v>23.215385</v>
+      </c>
+      <c r="F231" t="s">
+        <v>821</v>
+      </c>
+      <c r="G231" t="s">
         <v>822</v>
       </c>
-      <c r="B231" t="s">
-        <v>497</v>
-      </c>
-      <c r="C231" t="s">
-        <v>498</v>
-      </c>
-      <c r="D231" t="s">
+      <c r="H231" t="s">
         <v>823</v>
-      </c>
-      <c r="E231" t="n">
-        <v>1.2569776</v>
-      </c>
-      <c r="F231" t="s">
-        <v>824</v>
-      </c>
-      <c r="G231" t="s">
-        <v>820</v>
-      </c>
-      <c r="H231" t="s">
-        <v>825</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="s">
+        <v>824</v>
+      </c>
+      <c r="B232" t="s">
+        <v>801</v>
+      </c>
+      <c r="C232" t="s">
+        <v>819</v>
+      </c>
+      <c r="D232" t="s">
+        <v>825</v>
+      </c>
+      <c r="E232" t="n">
+        <v>8</v>
+      </c>
+      <c r="F232" t="s">
+        <v>117</v>
+      </c>
+      <c r="G232" t="s">
+        <v>822</v>
+      </c>
+      <c r="H232" t="s">
         <v>826</v>
-      </c>
-      <c r="B232" t="s">
-        <v>476</v>
-      </c>
-      <c r="C232" t="s">
-        <v>827</v>
-      </c>
-      <c r="D232" t="s">
-        <v>828</v>
-      </c>
-      <c r="E232" t="n">
-        <v>15</v>
-      </c>
-      <c r="F232" t="s">
-        <v>449</v>
-      </c>
-      <c r="G232" t="s">
-        <v>829</v>
-      </c>
-      <c r="H232" t="s">
-        <v>830</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="B233" t="s">
-        <v>476</v>
+        <v>497</v>
       </c>
       <c r="C233" t="s">
-        <v>832</v>
+        <v>567</v>
       </c>
       <c r="D233" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="E233" t="n">
-        <v>0.76351351</v>
+        <v>1.2232249</v>
       </c>
       <c r="F233" t="s">
-        <v>382</v>
+        <v>569</v>
       </c>
       <c r="G233" t="s">
-        <v>834</v>
+        <v>300</v>
       </c>
       <c r="H233" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>836</v>
+        <v>830</v>
       </c>
       <c r="B234" t="s">
-        <v>476</v>
+        <v>497</v>
       </c>
       <c r="C234" t="s">
+        <v>567</v>
+      </c>
+      <c r="D234" t="s">
+        <v>831</v>
+      </c>
+      <c r="E234" t="n">
+        <v>1.2569776</v>
+      </c>
+      <c r="F234" t="s">
         <v>832</v>
       </c>
-      <c r="D234" t="s">
-        <v>837</v>
-      </c>
-      <c r="E234" t="n">
-        <v>0.93194444</v>
-      </c>
-      <c r="F234" t="s">
-        <v>838</v>
-      </c>
       <c r="G234" t="s">
-        <v>834</v>
+        <v>300</v>
       </c>
       <c r="H234" t="s">
-        <v>839</v>
+        <v>829</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
       <c r="B235" t="s">
         <v>476</v>
       </c>
       <c r="C235" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="D235" t="s">
-        <v>841</v>
+        <v>835</v>
       </c>
       <c r="E235" t="n">
-        <v>0.5</v>
+        <v>15</v>
       </c>
       <c r="F235" t="s">
-        <v>842</v>
+        <v>449</v>
       </c>
       <c r="G235" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="H235" t="s">
-        <v>843</v>
+        <v>837</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>844</v>
+        <v>838</v>
       </c>
       <c r="B236" t="s">
         <v>476</v>
       </c>
       <c r="C236" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="D236" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="E236" t="n">
-        <v>0.54583333</v>
+        <v>0.76351351</v>
       </c>
       <c r="F236" t="s">
-        <v>846</v>
+        <v>382</v>
       </c>
       <c r="G236" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="H236" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="B237" t="s">
         <v>476</v>
       </c>
       <c r="C237" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="D237" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="E237" t="n">
-        <v>0.39354575</v>
+        <v>0.93194444</v>
       </c>
       <c r="F237" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="G237" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="H237" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="B238" t="s">
         <v>476</v>
       </c>
       <c r="C238" t="s">
-        <v>853</v>
+        <v>839</v>
       </c>
       <c r="D238" t="s">
-        <v>854</v>
+        <v>848</v>
       </c>
       <c r="E238" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="F238" t="s">
-        <v>855</v>
+        <v>849</v>
       </c>
       <c r="G238" t="s">
-        <v>856</v>
+        <v>841</v>
       </c>
       <c r="H238" t="s">
-        <v>857</v>
+        <v>850</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>858</v>
+        <v>851</v>
       </c>
       <c r="B239" t="s">
         <v>476</v>
       </c>
       <c r="C239" t="s">
+        <v>839</v>
+      </c>
+      <c r="D239" t="s">
+        <v>852</v>
+      </c>
+      <c r="E239" t="n">
+        <v>0.54583333</v>
+      </c>
+      <c r="F239" t="s">
         <v>853</v>
       </c>
-      <c r="D239" t="s">
-        <v>859</v>
-      </c>
-      <c r="E239" t="n">
-        <v>19</v>
-      </c>
-      <c r="F239" t="s">
-        <v>860</v>
-      </c>
       <c r="G239" t="s">
-        <v>856</v>
+        <v>841</v>
       </c>
       <c r="H239" t="s">
-        <v>861</v>
+        <v>854</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>862</v>
+        <v>855</v>
       </c>
       <c r="B240" t="s">
         <v>476</v>
       </c>
       <c r="C240" t="s">
-        <v>863</v>
+        <v>839</v>
       </c>
       <c r="D240" t="s">
-        <v>864</v>
+        <v>856</v>
       </c>
       <c r="E240" t="n">
-        <v>2375</v>
+        <v>0.39354575</v>
       </c>
       <c r="F240" t="s">
-        <v>865</v>
+        <v>857</v>
       </c>
       <c r="G240" t="s">
-        <v>866</v>
+        <v>841</v>
       </c>
       <c r="H240" t="s">
-        <v>867</v>
+        <v>858</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>868</v>
+        <v>859</v>
       </c>
       <c r="B241" t="s">
         <v>476</v>
       </c>
       <c r="C241" t="s">
+        <v>860</v>
+      </c>
+      <c r="D241" t="s">
+        <v>861</v>
+      </c>
+      <c r="E241" t="n">
+        <v>5</v>
+      </c>
+      <c r="F241" t="s">
+        <v>862</v>
+      </c>
+      <c r="G241" t="s">
         <v>863</v>
       </c>
-      <c r="D241" t="s">
-        <v>869</v>
-      </c>
-      <c r="E241" t="n">
-        <v>950</v>
-      </c>
-      <c r="F241" t="s">
-        <v>870</v>
-      </c>
-      <c r="G241" t="s">
-        <v>866</v>
-      </c>
       <c r="H241" t="s">
-        <v>871</v>
+        <v>864</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>872</v>
+        <v>865</v>
       </c>
       <c r="B242" t="s">
         <v>476</v>
       </c>
       <c r="C242" t="s">
+        <v>860</v>
+      </c>
+      <c r="D242" t="s">
+        <v>866</v>
+      </c>
+      <c r="E242" t="n">
+        <v>19</v>
+      </c>
+      <c r="F242" t="s">
+        <v>867</v>
+      </c>
+      <c r="G242" t="s">
         <v>863</v>
       </c>
-      <c r="D242" t="s">
-        <v>873</v>
-      </c>
-      <c r="E242" t="n">
-        <v>2308</v>
-      </c>
-      <c r="F242" t="s">
-        <v>874</v>
-      </c>
-      <c r="G242" t="s">
-        <v>866</v>
-      </c>
       <c r="H242" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>876</v>
+        <v>869</v>
       </c>
       <c r="B243" t="s">
         <v>476</v>
       </c>
       <c r="C243" t="s">
-        <v>877</v>
+        <v>870</v>
       </c>
       <c r="D243" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="E243" t="n">
-        <v>148</v>
+        <v>2375</v>
       </c>
       <c r="F243" t="s">
-        <v>39</v>
+        <v>872</v>
       </c>
       <c r="G243" t="s">
-        <v>834</v>
+        <v>873</v>
       </c>
       <c r="H243" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="B244" t="s">
         <v>476</v>
       </c>
       <c r="C244" t="s">
+        <v>870</v>
+      </c>
+      <c r="D244" t="s">
+        <v>876</v>
+      </c>
+      <c r="E244" t="n">
+        <v>950</v>
+      </c>
+      <c r="F244" t="s">
         <v>877</v>
       </c>
-      <c r="D244" t="s">
-        <v>881</v>
-      </c>
-      <c r="E244" t="n">
-        <v>720</v>
-      </c>
-      <c r="F244" t="s">
-        <v>882</v>
-      </c>
       <c r="G244" t="s">
-        <v>834</v>
+        <v>873</v>
       </c>
       <c r="H244" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="B245" t="s">
         <v>476</v>
       </c>
       <c r="C245" t="s">
-        <v>832</v>
+        <v>870</v>
       </c>
       <c r="D245" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="E245" t="n">
-        <v>0.0000000013458895</v>
+        <v>2308</v>
       </c>
       <c r="F245" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="G245" t="s">
-        <v>834</v>
+        <v>873</v>
       </c>
       <c r="H245" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="B246" t="s">
         <v>476</v>
       </c>
       <c r="C246" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="D246" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="E246" t="n">
-        <v>0.0000000000028256872</v>
+        <v>148</v>
       </c>
       <c r="F246" t="s">
-        <v>891</v>
+        <v>39</v>
       </c>
       <c r="G246" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="H246" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>893</v>
+        <v>887</v>
       </c>
       <c r="B247" t="s">
         <v>476</v>
       </c>
       <c r="C247" t="s">
-        <v>894</v>
+        <v>884</v>
       </c>
       <c r="D247" t="s">
-        <v>895</v>
+        <v>888</v>
       </c>
       <c r="E247" t="n">
-        <v>21</v>
+        <v>720</v>
       </c>
       <c r="F247" t="s">
-        <v>666</v>
+        <v>889</v>
       </c>
       <c r="G247" t="s">
-        <v>896</v>
+        <v>841</v>
       </c>
       <c r="H247" t="s">
-        <v>897</v>
+        <v>890</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>898</v>
+        <v>891</v>
       </c>
       <c r="B248" t="s">
-        <v>899</v>
+        <v>476</v>
       </c>
       <c r="C248" t="s">
-        <v>900</v>
+        <v>839</v>
       </c>
       <c r="D248" t="s">
-        <v>901</v>
+        <v>892</v>
       </c>
       <c r="E248" t="n">
-        <v>575</v>
+        <v>0.0000000013458895</v>
       </c>
       <c r="F248" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="G248" t="s">
-        <v>903</v>
+        <v>841</v>
       </c>
       <c r="H248" t="s">
-        <v>904</v>
+        <v>894</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>905</v>
+        <v>895</v>
       </c>
       <c r="B249" t="s">
+        <v>476</v>
+      </c>
+      <c r="C249" t="s">
+        <v>896</v>
+      </c>
+      <c r="D249" t="s">
+        <v>897</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0.0000000000028256872</v>
+      </c>
+      <c r="F249" t="s">
+        <v>898</v>
+      </c>
+      <c r="G249" t="s">
+        <v>841</v>
+      </c>
+      <c r="H249" t="s">
         <v>899</v>
-      </c>
-      <c r="C249" t="s">
-        <v>900</v>
-      </c>
-      <c r="D249" t="s">
-        <v>906</v>
-      </c>
-      <c r="E249" t="n">
-        <v>473</v>
-      </c>
-      <c r="F249" t="s">
-        <v>907</v>
-      </c>
-      <c r="G249" t="s">
-        <v>903</v>
-      </c>
-      <c r="H249" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>909</v>
+        <v>900</v>
       </c>
       <c r="B250" t="s">
-        <v>899</v>
+        <v>476</v>
       </c>
       <c r="C250" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="D250" t="s">
-        <v>910</v>
+        <v>902</v>
       </c>
       <c r="E250" t="n">
-        <v>281</v>
+        <v>21</v>
       </c>
       <c r="F250" t="s">
-        <v>911</v>
+        <v>676</v>
       </c>
       <c r="G250" t="s">
         <v>903</v>
       </c>
       <c r="H250" t="s">
-        <v>912</v>
+        <v>904</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>913</v>
+        <v>905</v>
       </c>
       <c r="B251" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C251" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D251" t="s">
-        <v>914</v>
+        <v>908</v>
       </c>
       <c r="E251" t="n">
-        <v>294</v>
+        <v>575</v>
       </c>
       <c r="F251" t="s">
-        <v>915</v>
+        <v>909</v>
       </c>
       <c r="G251" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H251" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="B252" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C252" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D252" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="E252" t="n">
-        <v>260</v>
+        <v>473</v>
       </c>
       <c r="F252" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="G252" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H252" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="B253" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C253" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D253" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="E253" t="n">
-        <v>12</v>
+        <v>281</v>
       </c>
       <c r="F253" t="s">
-        <v>619</v>
+        <v>918</v>
       </c>
       <c r="G253" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H253" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="B254" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C254" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D254" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="E254" t="n">
-        <v>248</v>
+        <v>294</v>
       </c>
       <c r="F254" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="G254" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H254" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="B255" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C255" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D255" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="E255" t="n">
-        <v>152</v>
+        <v>260</v>
       </c>
       <c r="F255" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="G255" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H255" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="B256" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C256" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D256" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="E256" t="n">
-        <v>149</v>
+        <v>12</v>
       </c>
       <c r="F256" t="s">
-        <v>45</v>
+        <v>629</v>
       </c>
       <c r="G256" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H256" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="B257" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C257" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D257" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="E257" t="n">
-        <v>87</v>
+        <v>248</v>
       </c>
       <c r="F257" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="G257" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H257" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
       <c r="B258" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C258" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D258" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="E258" t="n">
-        <v>9</v>
+        <v>152</v>
       </c>
       <c r="F258" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="G258" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H258" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="B259" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C259" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="D259" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="E259" t="n">
-        <v>13</v>
+        <v>149</v>
       </c>
       <c r="F259" t="s">
-        <v>945</v>
+        <v>45</v>
       </c>
       <c r="G259" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H259" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="B260" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C260" t="s">
-        <v>948</v>
+        <v>907</v>
       </c>
       <c r="D260" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="E260" t="n">
-        <v>11964</v>
+        <v>87</v>
       </c>
       <c r="F260" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="G260" t="s">
-        <v>951</v>
+        <v>910</v>
       </c>
       <c r="H260" t="s">
-        <v>952</v>
+        <v>945</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>953</v>
+        <v>946</v>
       </c>
       <c r="B261" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C261" t="s">
+        <v>907</v>
+      </c>
+      <c r="D261" t="s">
+        <v>947</v>
+      </c>
+      <c r="E261" t="n">
+        <v>9</v>
+      </c>
+      <c r="F261" t="s">
         <v>948</v>
       </c>
-      <c r="D261" t="s">
-        <v>954</v>
-      </c>
-      <c r="E261" t="n">
-        <v>10651</v>
-      </c>
-      <c r="F261" t="s">
-        <v>103</v>
-      </c>
       <c r="G261" t="s">
-        <v>951</v>
+        <v>910</v>
       </c>
       <c r="H261" t="s">
-        <v>104</v>
+        <v>949</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="B262" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C262" t="s">
-        <v>956</v>
+        <v>907</v>
       </c>
       <c r="D262" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="E262" t="n">
-        <v>341</v>
+        <v>13</v>
       </c>
       <c r="F262" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="G262" t="s">
-        <v>959</v>
+        <v>910</v>
       </c>
       <c r="H262" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>961</v>
+        <v>954</v>
       </c>
       <c r="B263" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C263" t="s">
+        <v>955</v>
+      </c>
+      <c r="D263" t="s">
         <v>956</v>
       </c>
-      <c r="D263" t="s">
-        <v>962</v>
-      </c>
       <c r="E263" t="n">
-        <v>219</v>
+        <v>11964</v>
       </c>
       <c r="F263" t="s">
-        <v>963</v>
+        <v>957</v>
       </c>
       <c r="G263" t="s">
+        <v>958</v>
+      </c>
+      <c r="H263" t="s">
         <v>959</v>
-      </c>
-      <c r="H263" t="s">
-        <v>960</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="B264" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C264" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D264" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="E264" t="n">
-        <v>203</v>
+        <v>10651</v>
       </c>
       <c r="F264" t="s">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="G264" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H264" t="s">
-        <v>960</v>
+        <v>104</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="s">
+        <v>962</v>
+      </c>
+      <c r="B265" t="s">
+        <v>906</v>
+      </c>
+      <c r="C265" t="s">
+        <v>963</v>
+      </c>
+      <c r="D265" t="s">
+        <v>964</v>
+      </c>
+      <c r="E265" t="n">
+        <v>341</v>
+      </c>
+      <c r="F265" t="s">
+        <v>965</v>
+      </c>
+      <c r="G265" t="s">
         <v>966</v>
       </c>
-      <c r="B265" t="s">
-        <v>899</v>
-      </c>
-      <c r="C265" t="s">
-        <v>956</v>
-      </c>
-      <c r="D265" t="s">
+      <c r="H265" t="s">
         <v>967</v>
-      </c>
-      <c r="E265" t="n">
-        <v>24</v>
-      </c>
-      <c r="F265" t="s">
-        <v>968</v>
-      </c>
-      <c r="G265" t="s">
-        <v>14</v>
-      </c>
-      <c r="H265" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="s">
+        <v>968</v>
+      </c>
+      <c r="B266" t="s">
+        <v>906</v>
+      </c>
+      <c r="C266" t="s">
+        <v>963</v>
+      </c>
+      <c r="D266" t="s">
+        <v>969</v>
+      </c>
+      <c r="E266" t="n">
+        <v>219</v>
+      </c>
+      <c r="F266" t="s">
         <v>970</v>
       </c>
-      <c r="B266" t="s">
-        <v>899</v>
-      </c>
-      <c r="C266" t="s">
-        <v>956</v>
-      </c>
-      <c r="D266" t="s">
-        <v>971</v>
-      </c>
-      <c r="E266" t="n">
-        <v>2</v>
-      </c>
-      <c r="F266" t="s">
-        <v>972</v>
-      </c>
       <c r="G266" t="s">
-        <v>14</v>
+        <v>966</v>
       </c>
       <c r="H266" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="B267" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C267" t="s">
-        <v>956</v>
+        <v>963</v>
       </c>
       <c r="D267" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="E267" t="n">
-        <v>0</v>
+        <v>203</v>
       </c>
       <c r="F267" t="s">
-        <v>975</v>
+        <v>28</v>
       </c>
       <c r="G267" t="s">
-        <v>14</v>
+        <v>966</v>
       </c>
       <c r="H267" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="s">
+        <v>973</v>
+      </c>
+      <c r="B268" t="s">
+        <v>906</v>
+      </c>
+      <c r="C268" t="s">
+        <v>963</v>
+      </c>
+      <c r="D268" t="s">
+        <v>974</v>
+      </c>
+      <c r="E268" t="n">
+        <v>24</v>
+      </c>
+      <c r="F268" t="s">
+        <v>975</v>
+      </c>
+      <c r="G268" t="s">
+        <v>14</v>
+      </c>
+      <c r="H268" t="s">
         <v>976</v>
-      </c>
-      <c r="B268" t="s">
-        <v>899</v>
-      </c>
-      <c r="C268" t="s">
-        <v>977</v>
-      </c>
-      <c r="D268" t="s">
-        <v>978</v>
-      </c>
-      <c r="E268" t="n">
-        <v>5</v>
-      </c>
-      <c r="F268" t="s">
-        <v>671</v>
-      </c>
-      <c r="G268" t="s">
-        <v>979</v>
-      </c>
-      <c r="H268" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="B269" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C269" t="s">
-        <v>977</v>
+        <v>963</v>
       </c>
       <c r="D269" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
       <c r="E269" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="F269" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="G269" t="s">
-        <v>979</v>
+        <v>14</v>
       </c>
       <c r="H269" t="s">
-        <v>984</v>
+        <v>976</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="B270" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C270" t="s">
-        <v>977</v>
+        <v>963</v>
       </c>
       <c r="D270" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="E270" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="F270" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
       <c r="G270" t="s">
-        <v>979</v>
+        <v>14</v>
       </c>
       <c r="H270" t="s">
-        <v>988</v>
+        <v>976</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>989</v>
+        <v>983</v>
       </c>
       <c r="B271" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C271" t="s">
-        <v>990</v>
+        <v>984</v>
       </c>
       <c r="D271" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="E271" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="F271" t="s">
-        <v>992</v>
+        <v>681</v>
       </c>
       <c r="G271" t="s">
-        <v>316</v>
+        <v>986</v>
       </c>
       <c r="H271" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="B272" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C272" t="s">
+        <v>984</v>
+      </c>
+      <c r="D272" t="s">
+        <v>989</v>
+      </c>
+      <c r="E272" t="n">
+        <v>24</v>
+      </c>
+      <c r="F272" t="s">
         <v>990</v>
       </c>
-      <c r="D272" t="s">
-        <v>995</v>
-      </c>
-      <c r="E272" t="n">
-        <v>10</v>
-      </c>
-      <c r="F272" t="s">
-        <v>78</v>
-      </c>
       <c r="G272" t="s">
-        <v>316</v>
+        <v>986</v>
       </c>
       <c r="H272" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="B273" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C273" t="s">
-        <v>997</v>
+        <v>984</v>
       </c>
       <c r="D273" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
       <c r="E273" t="n">
-        <v>298</v>
+        <v>95</v>
       </c>
       <c r="F273" t="s">
-        <v>999</v>
+        <v>994</v>
       </c>
       <c r="G273" t="s">
-        <v>1000</v>
+        <v>986</v>
       </c>
       <c r="H273" t="s">
-        <v>1001</v>
+        <v>995</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>1002</v>
+        <v>996</v>
       </c>
       <c r="B274" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="C274" t="s">
         <v>997</v>
       </c>
       <c r="D274" t="s">
-        <v>1003</v>
+        <v>998</v>
       </c>
       <c r="E274" t="n">
-        <v>191</v>
+        <v>25</v>
       </c>
       <c r="F274" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="G274" t="s">
+        <v>316</v>
+      </c>
+      <c r="H274" t="s">
         <v>1000</v>
-      </c>
-      <c r="H274" t="s">
-        <v>1001</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="B275" t="s">
-        <v>1006</v>
+        <v>906</v>
       </c>
       <c r="C275" t="s">
-        <v>313</v>
+        <v>997</v>
       </c>
       <c r="D275" t="s">
-        <v>1007</v>
+        <v>1002</v>
       </c>
       <c r="E275" t="n">
-        <v>3700</v>
+        <v>10</v>
       </c>
       <c r="F275" t="s">
-        <v>676</v>
+        <v>78</v>
       </c>
       <c r="G275" t="s">
         <v>316</v>
       </c>
       <c r="H275" t="s">
-        <v>1008</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>1009</v>
+        <v>1003</v>
       </c>
       <c r="B276" t="s">
+        <v>906</v>
+      </c>
+      <c r="C276" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D276" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E276" t="n">
+        <v>298</v>
+      </c>
+      <c r="F276" t="s">
         <v>1006</v>
       </c>
-      <c r="C276" t="s">
-        <v>313</v>
-      </c>
-      <c r="D276" t="s">
-        <v>1010</v>
-      </c>
-      <c r="E276" t="n">
-        <v>1480</v>
-      </c>
-      <c r="F276" t="s">
-        <v>1011</v>
-      </c>
       <c r="G276" t="s">
-        <v>316</v>
+        <v>1007</v>
       </c>
       <c r="H276" t="s">
-        <v>871</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="B277" t="s">
-        <v>1006</v>
+        <v>906</v>
       </c>
       <c r="C277" t="s">
-        <v>313</v>
+        <v>1004</v>
       </c>
       <c r="D277" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
       <c r="E277" t="n">
-        <v>3585</v>
+        <v>191</v>
       </c>
       <c r="F277" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="G277" t="s">
-        <v>316</v>
+        <v>1007</v>
       </c>
       <c r="H277" t="s">
-        <v>875</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="B278" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C278" t="s">
-        <v>1016</v>
+        <v>313</v>
       </c>
       <c r="D278" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="E278" t="n">
         <v>3700</v>
       </c>
       <c r="F278" t="s">
-        <v>676</v>
+        <v>686</v>
       </c>
       <c r="G278" t="s">
-        <v>1018</v>
+        <v>316</v>
       </c>
       <c r="H278" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>1020</v>
+        <v>1016</v>
       </c>
       <c r="B279" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C279" t="s">
-        <v>1016</v>
+        <v>313</v>
       </c>
       <c r="D279" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="E279" t="n">
-        <v>148</v>
+        <v>1480</v>
       </c>
       <c r="F279" t="s">
-        <v>39</v>
+        <v>1018</v>
       </c>
       <c r="G279" t="s">
-        <v>1018</v>
+        <v>316</v>
       </c>
       <c r="H279" t="s">
-        <v>1019</v>
+        <v>878</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="B280" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C280" t="s">
-        <v>1016</v>
+        <v>313</v>
       </c>
       <c r="D280" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="E280" t="n">
-        <v>3700</v>
+        <v>3585</v>
       </c>
       <c r="F280" t="s">
-        <v>676</v>
+        <v>1021</v>
       </c>
       <c r="G280" t="s">
-        <v>1018</v>
+        <v>316</v>
       </c>
       <c r="H280" t="s">
-        <v>1019</v>
+        <v>882</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B281" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C281" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D281" t="s">
         <v>1024</v>
       </c>
-      <c r="B281" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C281" t="s">
+      <c r="E281" t="n">
+        <v>3700</v>
+      </c>
+      <c r="F281" t="s">
+        <v>686</v>
+      </c>
+      <c r="G281" t="s">
         <v>1025</v>
       </c>
-      <c r="D281" t="s">
+      <c r="H281" t="s">
         <v>1026</v>
-      </c>
-      <c r="E281" t="n">
-        <v>148</v>
-      </c>
-      <c r="F281" t="s">
-        <v>39</v>
-      </c>
-      <c r="G281" t="s">
-        <v>1027</v>
-      </c>
-      <c r="H281" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="B282" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C282" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="D282" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="E282" t="n">
         <v>148</v>
@@ -10737,61 +10755,139 @@
         <v>39</v>
       </c>
       <c r="G282" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="H282" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="B283" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C283" t="s">
-        <v>753</v>
+        <v>1023</v>
       </c>
       <c r="D283" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="E283" t="n">
-        <v>29600</v>
+        <v>3700</v>
       </c>
       <c r="F283" t="s">
-        <v>1033</v>
+        <v>686</v>
       </c>
       <c r="G283" t="s">
-        <v>776</v>
+        <v>1025</v>
       </c>
       <c r="H283" t="s">
-        <v>15</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B284" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1032</v>
+      </c>
+      <c r="D284" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E284" t="n">
+        <v>148</v>
+      </c>
+      <c r="F284" t="s">
+        <v>39</v>
+      </c>
+      <c r="G284" t="s">
         <v>1034</v>
       </c>
-      <c r="B284" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C284" t="s">
+      <c r="H284" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B285" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1032</v>
+      </c>
+      <c r="D285" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E285" t="n">
+        <v>148</v>
+      </c>
+      <c r="F285" t="s">
+        <v>39</v>
+      </c>
+      <c r="G285" t="s">
+        <v>1034</v>
+      </c>
+      <c r="H285" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B286" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C286" t="s">
+        <v>763</v>
+      </c>
+      <c r="D286" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E286" t="n">
+        <v>29600</v>
+      </c>
+      <c r="F286" t="s">
+        <v>1040</v>
+      </c>
+      <c r="G286" t="s">
+        <v>786</v>
+      </c>
+      <c r="H286" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B287" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C287" t="s">
         <v>498</v>
       </c>
-      <c r="D284" t="s">
-        <v>1035</v>
-      </c>
-      <c r="E284" t="n">
+      <c r="D287" t="s">
+        <v>1042</v>
+      </c>
+      <c r="E287" t="n">
         <v>200</v>
       </c>
-      <c r="F284" t="s">
+      <c r="F287" t="s">
         <v>94</v>
       </c>
-      <c r="G284" t="s">
-        <v>1036</v>
-      </c>
-      <c r="H284" t="s">
+      <c r="G287" t="s">
+        <v>501</v>
+      </c>
+      <c r="H287" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>